<commit_message>
Updated script to include port detection and Excel export
</commit_message>
<xml_diff>
--- a/simulated_attention_log.xlsx
+++ b/simulated_attention_log.xlsx
@@ -453,81 +453,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-06-14 13:22:42</t>
+          <t>2025-07-26 14:26:23</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1923221032573154</v>
+        <v>0.1853426124110005</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04727286828014791</v>
+        <v>0.0511098920159045</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2458004955202661</v>
+        <v>0.2757589922309253</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-06-14 13:22:44</t>
+          <t>2025-07-26 14:26:25</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1947367569607006</v>
+        <v>0.1980741572259427</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04865030355183179</v>
+        <v>0.05134152191150011</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2498259923351287</v>
+        <v>0.2592035358400388</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-06-14 13:22:46</t>
+          <t>2025-07-26 14:26:27</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1906743642938908</v>
+        <v>0.1977735007921861</v>
       </c>
       <c r="C4" t="n">
-        <v>0.04460837982009769</v>
+        <v>0.04969726216578309</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2339505889283668</v>
+        <v>0.251283725912317</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-06-14 13:22:48</t>
+          <t>2025-07-26 14:26:29</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1907449096374725</v>
+        <v>0.190574657953641</v>
       </c>
       <c r="C5" t="n">
-        <v>0.05334513864222395</v>
+        <v>0.04647118355020854</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2796674298863918</v>
+        <v>0.24384765555509</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-06-14 13:22:50</t>
+          <t>2025-07-26 14:26:31</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1858687054552969</v>
+        <v>0.1974817999135489</v>
       </c>
       <c r="C6" t="n">
-        <v>0.04789540080128126</v>
+        <v>0.04719279239861143</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2576840500608131</v>
+        <v>0.2389728694961809</v>
       </c>
     </row>
   </sheetData>

</xml_diff>